<commit_message>
Thanksgiving: Paradise's tax and add-on prices quoted, DAN out of the fee, posted fee 1,250; Blue Ocean full quote filed and compared with RSDS
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/thanksgiving_group_budget.xlsx
+++ b/december-plan/pricing/thanksgiving_group_budget.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="143">
   <si>
     <t xml:space="preserve">Thanksgiving (Puerto Rico) group budget — inputs (blue cells are editable)</t>
   </si>
@@ -76,10 +76,10 @@
     <t xml:space="preserve">Group discount</t>
   </si>
   <si>
-    <t xml:space="preserve">Puerto Rico sales tax on services (IVU)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INFERRED; Paradise said 'plus tax', rate asked</t>
+    <t xml:space="preserve">Puerto Rico sales tax (IVU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 24 Sep (Edwin, Paradise Scuba)</t>
   </si>
   <si>
     <t xml:space="preserve">Boat mornings (Thu, Fri, Sat; Sat out of the water by noon)</t>
@@ -97,15 +97,18 @@
     <t xml:space="preserve">USD/day</t>
   </si>
   <si>
-    <t xml:space="preserve">Night dive (optional add-on)</t>
+    <t xml:space="preserve">Night dive, single tank with lights, list price (optional add-on; group discount and tax apply)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 24 Sep; gear rental 25 extra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional third dive, one tank (add-on)</t>
   </si>
   <si>
     <t xml:space="preserve">INFERRED; asked</t>
   </si>
   <si>
-    <t xml:space="preserve">Optional third dive, one tank (add-on)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Paradise Scuba deposit</t>
   </si>
   <si>
@@ -160,16 +163,16 @@
     <t xml:space="preserve">Included for everyone</t>
   </si>
   <si>
-    <t xml:space="preserve">DAN membership + Preferred plan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tax buffer per head (hotel room tax and anything the quotes leave out)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">policy; PR room tax 9–11% plus fees</t>
+    <t xml:space="preserve">DAN cover inside the fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George 24 Sep: not in the fee; each diver buys their own cover (see own spending)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hotel room-tax buffer per head (PR room tax 9% plus fees; kept until the hotel quotes an all-in rate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">policy; diving tax is now inside the diving line</t>
   </si>
   <si>
     <t xml:space="preserve">Leader costs carried by the group</t>
@@ -193,7 +196,10 @@
     <t xml:space="preserve">half a room</t>
   </si>
   <si>
-    <t xml:space="preserve">George's DAN</t>
+    <t xml:space="preserve">George's DAN carried by the group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George 24 Sep: own cost like everyone</t>
   </si>
   <si>
     <t xml:space="preserve">George's gear</t>
@@ -211,7 +217,16 @@
     <t xml:space="preserve">Tips</t>
   </si>
   <si>
-    <t xml:space="preserve">Bioluminescent bay boat tour (optional add-on)</t>
+    <t xml:space="preserve">Sunset Bio Bay Cruise, list price (optional add-on; eat, cruise, swim; discount and tax apply)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 24 Sep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dive-accident cover, required, bought by each person</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADVERTISED: DAN membership 40 + Master 44</t>
   </si>
   <si>
     <t xml:space="preserve">Trip fee per certified diver, set at the pricing headcount (USD, 2 sharing)</t>
@@ -226,7 +241,7 @@
     <t xml:space="preserve">Gear rental, everyone</t>
   </si>
   <si>
-    <t xml:space="preserve">DAN dive-accident cover</t>
+    <t xml:space="preserve">DAN dive-accident cover (not in the fee; each person buys their own, see below)</t>
   </si>
   <si>
     <t xml:space="preserve">Hotel, 4 nights, 2 sharing</t>
@@ -253,10 +268,10 @@
     <t xml:space="preserve">Optional add-ons, charged at cost</t>
   </si>
   <si>
-    <t xml:space="preserve">Bio bay night tour</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Night dive</t>
+    <t xml:space="preserve">Sunset Bio Bay Cruise, after discount and tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Night dive, after discount and tax, plus gear</t>
   </si>
   <si>
     <t xml:space="preserve">Third dive in the afternoon</t>
@@ -268,7 +283,7 @@
     <t xml:space="preserve">Trip fee</t>
   </si>
   <si>
-    <t xml:space="preserve">Own spending: meals incl. Thanksgiving dinner, drinks, tips</t>
+    <t xml:space="preserve">Own spending: dive cover, meals incl. Thanksgiving dinner, drinks, tips</t>
   </si>
   <si>
     <t xml:space="preserve">Guidance budget</t>
@@ -844,7 +859,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="72"/>
@@ -988,12 +1003,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B12" s="7" t="n">
-        <v>95</v>
+        <v>140</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>14</v>
@@ -1013,12 +1028,12 @@
         <v>14</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B14" s="6" t="n">
         <v>0.5</v>
@@ -1027,12 +1042,12 @@
         <v>10</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -1040,7 +1055,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B16" s="7" t="n">
         <v>150</v>
@@ -1049,24 +1064,24 @@
         <v>14</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B17" s="5" t="n">
         <v>4</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B18" s="6" t="n">
         <v>0.25</v>
@@ -1075,12 +1090,12 @@
         <v>10</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -1088,7 +1103,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B20" s="7" t="n">
         <v>70</v>
@@ -1097,12 +1112,12 @@
         <v>23</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B21" s="5" t="n">
         <v>5</v>
@@ -1111,12 +1126,12 @@
         <v>20</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B22" s="7" t="n">
         <v>60</v>
@@ -1125,12 +1140,12 @@
         <v>14</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B23" s="5" t="n">
         <v>4</v>
@@ -1139,34 +1154,34 @@
         <v>7</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B25" s="7" t="n">
-        <v>119</v>
+        <v>0</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B26" s="7" t="n">
         <v>80</v>
@@ -1175,12 +1190,12 @@
         <v>14</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -1188,7 +1203,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B28" s="7" t="n">
         <v>550</v>
@@ -1197,12 +1212,12 @@
         <v>14</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B29" s="7" t="n">
         <f aca="false">Inputs!$B$16*Inputs!$B$17/2</f>
@@ -1212,12 +1227,12 @@
         <v>14</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B30" s="7" t="n">
         <f aca="false">Inputs!$B$29</f>
@@ -1227,24 +1242,26 @@
         <v>14</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B31" s="7" t="n">
-        <v>119</v>
+        <v>0</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D31" s="2"/>
+      <c r="D31" s="2" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B32" s="7" t="n">
         <f aca="false">Inputs!$B$11*Inputs!$B$10</f>
@@ -1254,12 +1271,12 @@
         <v>14</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -1267,7 +1284,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B34" s="7" t="n">
         <v>45</v>
@@ -1276,12 +1293,12 @@
         <v>23</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B35" s="5" t="n">
         <v>4</v>
@@ -1293,7 +1310,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B36" s="7" t="n">
         <v>40</v>
@@ -1302,21 +1319,35 @@
         <v>14</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B37" s="7" t="n">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>46</v>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>84</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1344,19 +1375,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B3" s="8" t="n">
         <f aca="false">ROUND(Inputs!$B$7*(1-Inputs!$B$8)*(1+Inputs!$B$9)*Inputs!$B$10,0)</f>
@@ -1365,25 +1396,25 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">Inputs!$B$11*Inputs!$B$10</f>
         <v>75</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">Inputs!$B$25</f>
-        <v>119</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">Inputs!$B$16*Inputs!$B$17/2</f>
@@ -1392,7 +1423,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">(ROUNDUP(Inputs!$B$4/Inputs!$B$23,0)*(Inputs!$B$20*Inputs!$B$21+Inputs!$B$22))/(Inputs!$B$4-1)</f>
@@ -1401,7 +1432,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">Inputs!$B$26</f>
@@ -1410,38 +1441,38 @@
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">(Inputs!$B$28+Inputs!$B$29+Inputs!$B$30+Inputs!$B$31+Inputs!$B$32)/(Inputs!$B$4-1)</f>
-        <v>149.333333333333</v>
+        <v>136.111111111111</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">SUM(B3:B9)</f>
-        <v>1272</v>
+        <v>1139.77777777778</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">ROUND(B10*Inputs!$B$5,0)</f>
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B12" s="9" t="n">
         <f aca="false">CEILING(B10+B11,50)</f>
-        <v>1350</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1450,31 +1481,31 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B14" s="8"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B15" s="8" t="n">
-        <f aca="false">Inputs!$B$37</f>
-        <v>45</v>
+        <f aca="false">ROUND(Inputs!$B$37*(1-Inputs!$B$8)*(1+Inputs!$B$9),0)</f>
+        <v>81</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B16" s="8" t="n">
-        <f aca="false">Inputs!$B$12</f>
-        <v>95</v>
+        <f aca="false">ROUND(Inputs!$B$12*(1-Inputs!$B$8)*(1+Inputs!$B$9),0)+Inputs!$B$11</f>
+        <v>158</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">Inputs!$B$13</f>
@@ -1487,44 +1518,44 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="B19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">B12</f>
-        <v>1350</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B21" s="8" t="n">
-        <f aca="false">Inputs!$B$34*Inputs!$B$35+Inputs!$B$36</f>
-        <v>220</v>
+        <f aca="false">Inputs!$B$38+Inputs!$B$34*Inputs!$B$35+Inputs!$B$36</f>
+        <v>304</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B22" s="9" t="n">
         <f aca="false">B20+B21</f>
-        <v>1570</v>
+        <v>1554</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B23" s="9" t="n">
         <f aca="false">B22+B15+B16</f>
-        <v>1710</v>
+        <v>1793</v>
       </c>
     </row>
   </sheetData>
@@ -1552,7 +1583,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1561,18 +1592,18 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B3" s="10" t="n">
         <v>8</v>
@@ -1586,7 +1617,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B4" s="10" t="n">
         <f aca="false">B3-1</f>
@@ -1603,7 +1634,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">ROUNDUP(B3/2,0)</f>
@@ -1620,7 +1651,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B6" s="10" t="n">
         <f aca="false">ROUNDUP(B3/Inputs!$B$23,0)</f>
@@ -1637,7 +1668,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -1645,24 +1676,24 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">B4*Fee!$B$12</f>
-        <v>9450</v>
+        <v>8750</v>
       </c>
       <c r="C8" s="9" t="n">
         <f aca="false">C4*Fee!$B$12</f>
-        <v>12150</v>
+        <v>11250</v>
       </c>
       <c r="D8" s="9" t="n">
         <f aca="false">D4*Fee!$B$12</f>
-        <v>14850</v>
+        <v>13750</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -1670,7 +1701,7 @@
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">ROUND(B4*Inputs!$B$7*(1-Inputs!$B$8)*(1+Inputs!$B$9)*Inputs!$B$10,0)</f>
@@ -1687,7 +1718,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">B3*Inputs!$B$11*Inputs!$B$10</f>
@@ -1704,24 +1735,24 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">B3*Inputs!$B$25</f>
-        <v>952</v>
+        <v>0</v>
       </c>
       <c r="C12" s="8" t="n">
         <f aca="false">C3*Inputs!$B$25</f>
-        <v>1190</v>
+        <v>0</v>
       </c>
       <c r="D12" s="8" t="n">
         <f aca="false">D3*Inputs!$B$25</f>
-        <v>1428</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B13" s="8" t="n">
         <f aca="false">B5*Inputs!$B$16*Inputs!$B$17</f>
@@ -1738,7 +1769,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">B6*(Inputs!$B$20*Inputs!$B$21+Inputs!$B$22)</f>
@@ -1755,7 +1786,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">B3*Inputs!$B$26</f>
@@ -1772,7 +1803,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">Inputs!$B$28</f>
@@ -1789,24 +1820,24 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B17" s="9" t="n">
         <f aca="false">B10+B11+B12+B13+B14+B15+B16</f>
-        <v>8848</v>
+        <v>7896</v>
       </c>
       <c r="C17" s="9" t="n">
         <f aca="false">C10+C11+C12+C13+C14+C15+C16</f>
-        <v>11230</v>
+        <v>10040</v>
       </c>
       <c r="D17" s="9" t="n">
         <f aca="false">D10+D11+D12+D13+D14+D15+D16</f>
-        <v>13203</v>
+        <v>11775</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -1814,24 +1845,24 @@
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="B19" s="9" t="n">
         <f aca="false">B8-B17</f>
-        <v>602</v>
+        <v>854</v>
       </c>
       <c r="C19" s="9" t="n">
         <f aca="false">C8-C17</f>
-        <v>920</v>
+        <v>1210</v>
       </c>
       <c r="D19" s="9" t="n">
         <f aca="false">D8-D17</f>
-        <v>1647</v>
+        <v>1975</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B20" s="11" t="str">
         <f aca="false">IF(B19&gt;=0,"yes","NO")</f>
@@ -1848,7 +1879,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -1856,7 +1887,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">B4*400</f>
@@ -1873,7 +1904,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">B10*Inputs!$B$14+B13*Inputs!$B$18</f>
@@ -1890,7 +1921,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B24" s="9" t="n">
         <f aca="false">B22-B23</f>
@@ -1907,41 +1938,41 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">B8-B22</f>
-        <v>6650</v>
+        <v>5950</v>
       </c>
       <c r="C25" s="8" t="n">
         <f aca="false">C8-C22</f>
-        <v>8550</v>
+        <v>7650</v>
       </c>
       <c r="D25" s="8" t="n">
         <f aca="false">D8-D22</f>
-        <v>10450</v>
+        <v>9350</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">B10*(1-Inputs!$B$14)+B13*(1-Inputs!$B$18)+B11+B12+B14</f>
-        <v>5615</v>
+        <v>4663</v>
       </c>
       <c r="C26" s="8" t="n">
         <f aca="false">C10*(1-Inputs!$B$14)+C13*(1-Inputs!$B$18)+C11+C12+C14</f>
-        <v>7275</v>
+        <v>6085</v>
       </c>
       <c r="D26" s="8" t="n">
         <f aca="false">D10*(1-Inputs!$B$14)+D13*(1-Inputs!$B$18)+D11+D12+D14</f>
-        <v>8525.5</v>
+        <v>7097.5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -1973,97 +2004,97 @@
   <sheetData>
     <row r="1" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2073,10 +2104,10 @@
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>11</v>
@@ -2084,10 +2115,10 @@
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
Thanksgiving: Nautilus quoted 176.70 a room tax included; budget rebuilt (1,200 three mornings / 1,050 two)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/thanksgiving_group_budget.xlsx
+++ b/december-plan/pricing/thanksgiving_group_budget.xlsx
@@ -118,10 +118,10 @@
     <t xml:space="preserve">Lodging (Parador Villa Parguera; QUOTE NEEDED, chased 24 Sep)</t>
   </si>
   <si>
-    <t xml:space="preserve">Room per night, 2 sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED band 135–170</t>
+    <t xml:space="preserve">Room per night, 2 sharing (Nautilus Hotel, tax included)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 30 Sep (Nautilus by La Jamaca: 155 + tax; grab-and-go breakfast optional, price to confirm)</t>
   </si>
   <si>
     <t xml:space="preserve">Nights (Wed 25 – Sun 29 Nov)</t>
@@ -169,10 +169,10 @@
     <t xml:space="preserve">George 24 Sep: not in the fee; each diver buys their own cover (see own spending)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hotel room-tax buffer per head (PR room tax 9% plus fees; kept until the hotel quotes an all-in rate)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">policy; diving tax is now inside the diving line</t>
+    <t xml:space="preserve">Hotel room-tax buffer per head</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zero: the Nautilus rate is quoted tax-inclusive (30 Sep)</t>
   </si>
   <si>
     <t xml:space="preserve">Leader costs carried by the group</t>
@@ -1053,12 +1053,12 @@
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B16" s="7" t="n">
-        <v>150</v>
+        <v>176.7</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>14</v>
@@ -1179,12 +1179,12 @@
         <v>47</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
         <v>48</v>
       </c>
       <c r="B26" s="7" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>14</v>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="B29" s="7" t="n">
         <f aca="false">Inputs!$B$16*Inputs!$B$17/2</f>
-        <v>300</v>
+        <v>353.4</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>14</v>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="B30" s="7" t="n">
         <f aca="false">Inputs!$B$29</f>
-        <v>300</v>
+        <v>353.4</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>14</v>
@@ -1418,7 +1418,7 @@
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">Inputs!$B$16*Inputs!$B$17/2</f>
-        <v>300</v>
+        <v>353.4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">Inputs!$B$26</f>
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">(Inputs!$B$28+Inputs!$B$29+Inputs!$B$30+Inputs!$B$31+Inputs!$B$32)/(Inputs!$B$4-1)</f>
-        <v>136.111111111111</v>
+        <v>147.977777777778</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">SUM(B3:B9)</f>
-        <v>1139.77777777778</v>
+        <v>1125.04444444444</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="B12" s="9" t="n">
         <f aca="false">CEILING(B10+B11,50)</f>
-        <v>1250</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">B12</f>
-        <v>1250</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="B22" s="9" t="n">
         <f aca="false">B20+B21</f>
-        <v>1554</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1555,7 +1555,7 @@
       </c>
       <c r="B23" s="9" t="n">
         <f aca="false">B22+B15+B16</f>
-        <v>1793</v>
+        <v>1743</v>
       </c>
     </row>
   </sheetData>
@@ -1680,15 +1680,15 @@
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">B4*Fee!$B$12</f>
-        <v>8750</v>
+        <v>8400</v>
       </c>
       <c r="C8" s="9" t="n">
         <f aca="false">C4*Fee!$B$12</f>
-        <v>11250</v>
+        <v>10800</v>
       </c>
       <c r="D8" s="9" t="n">
         <f aca="false">D4*Fee!$B$12</f>
-        <v>13750</v>
+        <v>13200</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1756,15 +1756,15 @@
       </c>
       <c r="B13" s="8" t="n">
         <f aca="false">B5*Inputs!$B$16*Inputs!$B$17</f>
-        <v>2400</v>
+        <v>2827.2</v>
       </c>
       <c r="C13" s="8" t="n">
         <f aca="false">C5*Inputs!$B$16*Inputs!$B$17</f>
-        <v>3000</v>
+        <v>3534</v>
       </c>
       <c r="D13" s="8" t="n">
         <f aca="false">D5*Inputs!$B$16*Inputs!$B$17</f>
-        <v>3600</v>
+        <v>4240.8</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1790,15 +1790,15 @@
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">B3*Inputs!$B$26</f>
-        <v>640</v>
+        <v>0</v>
       </c>
       <c r="C15" s="8" t="n">
         <f aca="false">C3*Inputs!$B$26</f>
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="D15" s="8" t="n">
         <f aca="false">D3*Inputs!$B$26</f>
-        <v>960</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1824,15 +1824,15 @@
       </c>
       <c r="B17" s="9" t="n">
         <f aca="false">B10+B11+B12+B13+B14+B15+B16</f>
-        <v>7896</v>
+        <v>7683.2</v>
       </c>
       <c r="C17" s="9" t="n">
         <f aca="false">C10+C11+C12+C13+C14+C15+C16</f>
-        <v>10040</v>
+        <v>9774</v>
       </c>
       <c r="D17" s="9" t="n">
         <f aca="false">D10+D11+D12+D13+D14+D15+D16</f>
-        <v>11775</v>
+        <v>11455.8</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1849,15 +1849,15 @@
       </c>
       <c r="B19" s="9" t="n">
         <f aca="false">B8-B17</f>
-        <v>854</v>
+        <v>716.8</v>
       </c>
       <c r="C19" s="9" t="n">
         <f aca="false">C8-C17</f>
-        <v>1210</v>
+        <v>1026</v>
       </c>
       <c r="D19" s="9" t="n">
         <f aca="false">D8-D17</f>
-        <v>1975</v>
+        <v>1744.2</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1908,15 +1908,15 @@
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">B10*Inputs!$B$14+B13*Inputs!$B$18</f>
-        <v>2043</v>
+        <v>2149.8</v>
       </c>
       <c r="C23" s="8" t="n">
         <f aca="false">C10*Inputs!$B$14+C13*Inputs!$B$18</f>
-        <v>2605</v>
+        <v>2738.5</v>
       </c>
       <c r="D23" s="8" t="n">
         <f aca="false">D10*Inputs!$B$14+D13*Inputs!$B$18</f>
-        <v>3167.5</v>
+        <v>3327.7</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1925,15 +1925,15 @@
       </c>
       <c r="B24" s="9" t="n">
         <f aca="false">B22-B23</f>
-        <v>757</v>
+        <v>650.2</v>
       </c>
       <c r="C24" s="9" t="n">
         <f aca="false">C22-C23</f>
-        <v>995</v>
+        <v>861.5</v>
       </c>
       <c r="D24" s="9" t="n">
         <f aca="false">D22-D23</f>
-        <v>1232.5</v>
+        <v>1072.3</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1942,15 +1942,15 @@
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">B8-B22</f>
-        <v>5950</v>
+        <v>5600</v>
       </c>
       <c r="C25" s="8" t="n">
         <f aca="false">C8-C22</f>
-        <v>7650</v>
+        <v>7200</v>
       </c>
       <c r="D25" s="8" t="n">
         <f aca="false">D8-D22</f>
-        <v>9350</v>
+        <v>8800</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1959,15 +1959,15 @@
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">B10*(1-Inputs!$B$14)+B13*(1-Inputs!$B$18)+B11+B12+B14</f>
-        <v>4663</v>
+        <v>4983.4</v>
       </c>
       <c r="C26" s="8" t="n">
         <f aca="false">C10*(1-Inputs!$B$14)+C13*(1-Inputs!$B$18)+C11+C12+C14</f>
-        <v>6085</v>
+        <v>6485.5</v>
       </c>
       <c r="D26" s="8" t="n">
         <f aca="false">D10*(1-Inputs!$B$14)+D13*(1-Inputs!$B$18)+D11+D12+D14</f>
-        <v>7097.5</v>
+        <v>7578.1</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>